<commit_message>
Rewrite explanations that referenced choice letters (ア/イ/ウ/エ)
Answer choices display in randomized order and use circled-number
labels (①②③④), so explanations saying things like "正解はウとなる"
no longer correspond to what the user sees. Rewrote 24 explanations
to state the actual answer content instead of the original letter.
</commit_message>
<xml_diff>
--- a/db/sample-data/study-materials-sample.xlsx
+++ b/db/sample-data/study-materials-sample.xlsx
@@ -8508,7 +8508,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>電子メールの送信にはSMTP(Simple Mail Transfer Protocol)が用いられ、受信にはPOP3やIMAP4が用いられる。したがって、送信プロトコルにSMTP、受信プロトコルにIMAP4を挙げているエが正しい組合せである。</t>
+          <t>電子メールの送信にはSMTP(Simple Mail Transfer Protocol)が用いられ、受信にはPOP3やIMAP4が用いられる。したがって、送信プロトコルにSMTP、受信プロトコルにIMAP4を挙げている組合せが正しい。</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -11407,7 +11407,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>偽装請負とは，形式上は請負契約でありながら，実態として発注元が請負元の労働者に直接指揮命令を行っている状態を指す。指揮命令の所在がポイントであり，作業場所がどちらの企業内かは偽装請負の判定に直接関係しない。aはA社内でA社の責任者が指揮命令しており偽装請負に該当する。cはB社内であってもA社の責任者が指揮命令しているため偽装請負に該当する。bはA社内での作業だが，指揮命令はB社の責任者が行っており，請負契約の本来の形態であるため偽装請負ではない。したがって，偽装請負に該当するのはaとcであり，正解はウとなる。</t>
+          <t>偽装請負とは，形式上は請負契約でありながら，実態として発注元が請負元の労働者に直接指揮命令を行っている状態を指す。指揮命令の所在がポイントであり，作業場所がどちらの企業内かは偽装請負の判定に直接関係しない。aはA社内でA社の責任者が指揮命令しており偽装請負に該当する。cはB社内であってもA社の責任者が指揮命令しているため偽装請負に該当する。bはA社内での作業だが，指揮命令はB社の責任者が行っており，請負契約の本来の形態であるため偽装請負ではない。したがって，偽装請負に該当するのはaとcであり，「a, c」を挙げている選択肢が正解となる。</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -11492,7 +11492,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>ISO/IEC 27017は，情報セキュリティマネジメントシステムの国際規格ISO/IEC 27001（及びJIS Q 27001）を基礎とし，クラウドサービスに特化した情報セキュリティ管理策のガイドラインとして追加制定された規格である。したがって正解はウとなる。</t>
+          <t>ISO/IEC 27017は，情報セキュリティマネジメントシステムの国際規格ISO/IEC 27001（及びJIS Q 27001）を基礎とし，クラウドサービスに特化した情報セキュリティ管理策のガイドラインとして追加制定された規格である。したがって正解は「ISO/IEC 27017」である。</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -11578,7 +11578,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>官民データ活用推進基本法における「官民データ」とは，国や地方公共団体が保有するデータに加え，独立行政法人や事業者（民間企業や大学等）が事業活動に伴って取得・利用するデータを幅広く含む概念である。県庁（地方公共団体），大学，電力事業者，独立行政法人はいずれも官民データを所有する組織体に該当する。したがって，a，b，c，dの全てが該当し，正解はイとなる。</t>
+          <t>官民データ活用推進基本法における「官民データ」とは，国や地方公共団体が保有するデータに加え，独立行政法人や事業者（民間企業や大学等）が事業活動に伴って取得・利用するデータを幅広く含む概念である。県庁（地方公共団体），大学，電力事業者，独立行政法人はいずれも官民データを所有する組織体に該当する。したがって，a，b，c，dの全てが該当し，「a, b, c, d」を挙げている選択肢が正解となる。</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -11663,7 +11663,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>VRIO分析は，Value（経済価値），Rarity（希少性），Imitability（模倣困難性），Organization（組織）の四つの要素の頭文字を取った分析フレームワークであり，自社の経営資源が競争優位の源泉になり得るかを評価する手法である。したがって正解はエとなる。</t>
+          <t>VRIO分析は，Value（経済価値），Rarity（希少性），Imitability（模倣困難性），Organization（組織）の四つの要素の頭文字を取った分析フレームワークであり，自社の経営資源が競争優位の源泉になり得るかを評価する手法である。したがって正解は「VRIO分析」である。</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -11748,7 +11748,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>仕入単価が期首から期末にかけて上昇し続けた場合，期末の仕入単価は期中平均値よりも高い。期末棚卸高の計算に期末の仕入単価（平均より高い値）を用いると，期末棚卸高は平均値を用いた場合より高くなる。売上原価は「期首棚卸高＋当期商品仕入高－期末棚卸高」で計算されるため，期末棚卸高が大きくなるほど売上原価は小さくなる。したがって，期末棚卸高は上がり，売上原価は下がることになり，正解はウとなる。</t>
+          <t>仕入単価が期首から期末にかけて上昇し続けた場合，期末の仕入単価は期中平均値よりも高い。期末棚卸高の計算に期末の仕入単価（平均より高い値）を用いると，期末棚卸高は平均値を用いた場合より高くなる。売上原価は「期首棚卸高＋当期商品仕入高－期末棚卸高」で計算されるため，期末棚卸高が大きくなるほど売上原価は小さくなる。したがって，「期末棚卸高は上がり，売上原価は下がる」が正解となる。</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -11833,7 +11833,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>特定電子メール法は，原則として事前に受信者の同意（オプトイン）を得ていない広告宣伝メールの送信を規制している。イは，受信者の事前同意を得ずに広告宣伝メールを送信し，拒否通知があった場合のみ送信をやめればよいと誤って考えている点が規制対象となる行為に該当する。アは公表されているメールアドレス宛ての送信で一定の例外規定に該当し得る。ウは広告宣伝メールではなく取引に関する事務連絡・料金請求メールであるため規制対象外。エは既存の取引関係がある相手への自社製品に関する広告であり，法律上の例外（取引関係にある者への通知）に該当し得る。したがって，規制対象となり得るのはイであり，正解はイとなる。</t>
+          <t>特定電子メール法は，原則として事前に受信者の同意（オプトイン）を得ていない広告宣伝メールの送信を規制している。受信者の事前同意を得ずに広告宣伝メールを送信し，拒否通知があった場合のみ送信をやめればよいと考えて送信する行為は，この規制対象となる。公表されているメールアドレス宛ての送信は一定の例外規定に該当し得る。事務連絡・料金請求メールは広告宣伝メールに当たらないため規制対象外。既存の取引関係がある相手への自社製品に関する広告は，法律上の例外（取引関係にある者への通知）に該当し得る。したがって，受信者からの拒否通知があった場合にのみ送信をやめればよいと考えて送信した事例が正解となる。</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -11918,7 +11918,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>PoC（Proof of Concept）は，新しい概念やアイディアが実現可能かどうかを検証するために，開発の前段階で行う実証・試作のことである。したがって正解はイとなる。</t>
+          <t>PoC（Proof of Concept）は，新しい概念やアイディアが実現可能かどうかを検証するために，開発の前段階で行う実証・試作のことである。したがって正解は「PoC」である。</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -12007,7 +12007,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>機械学習のバイアス低減やデータ品質確保のためには，学習目的への適合性確認（a），データの出所・信頼性の確認（b），学習目的に合わせた適切なアノテーション付与（c），人間でも判定困難な低品質データの除外（d）のいずれもが有効な対策である。したがって，a，b，c，dの全てが適切であり，正解はイとなる。</t>
+          <t>機械学習のバイアス低減やデータ品質確保のためには，学習目的への適合性確認（a），データの出所・信頼性の確認（b），学習目的に合わせた適切なアノテーション付与（c），人間でも判定困難な低品質データの除外（d）のいずれもが有効な対策である。したがって，a，b，c，dの全てが適切であり，「a, b, c, d」を挙げている選択肢が正解となる。</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -12092,7 +12092,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>ハッカソンとは，プログラマーやデザイナーなどのエンジニアが複数のチームに分かれ，与えられたテーマに基づき，短期間（数時間から数日程度）でソフトウェアやサービスのプロトタイプを作成し，その成果を競い合うイベントである。したがって正解はウとなる。</t>
+          <t>ハッカソンとは，プログラマーやデザイナーなどのエンジニアが複数のチームに分かれ，与えられたテーマに基づき，短期間（数時間から数日程度）でソフトウェアやサービスのプロトタイプを作成し，その成果を競い合うイベントである。したがって正解は，複数の参加チームがプロトタイプを短期間で作成し成果を発表して競い合うと説明している選択肢である。</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -12177,7 +12177,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>ハルシネーション（Hallucination）とは，生成AIがもっともらしいが事実に基づかない誤った内容を，あたかも真実であるかのように出力する現象を指す用語である。したがって正解はエとなる。</t>
+          <t>ハルシネーション（Hallucination）とは，生成AIがもっともらしいが事実に基づかない誤った内容を，あたかも真実であるかのように出力する現象を指す用語である。したがって正解は「ハルシネーション」である。</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -12262,7 +12262,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>FMS（Flexible Manufacturing System：フレキシブル生産システム）とは，複数の工作機械や産業用ロボットなどをコンピュータで有機的に結合し，多品種少量生産に柔軟に対応できるよう生産プロセス全体を統括的に制御・管理する仕組みである。したがって正解はエとなる。</t>
+          <t>FMS（Flexible Manufacturing System：フレキシブル生産システム）とは，複数の工作機械や産業用ロボットなどをコンピュータで有機的に結合し，多品種少量生産に柔軟に対応できるよう生産プロセス全体を統括的に制御・管理する仕組みである。したがって正解は，複数の工作機械や産業用ロボットなどを有機的に結合し，生産プロセス全体を統括的に制御・管理すると説明している選択肢である。</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -12347,7 +12347,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>サービスマーク（役務商標）とは，商標法において，運輸業，金融業などのサービス（役務）を提供する事業者が，自社の役務を他社の役務と区別するために使用する商標のことである。したがって正解はエとなる。</t>
+          <t>サービスマーク（役務商標）とは，商標法において，運輸業，金融業などのサービス（役務）を提供する事業者が，自社の役務を他社の役務と区別するために使用する商標のことである。したがって正解は，輸送業者，金融業者などが提供する役務を他社の役務と区別するために表示する商標と説明している選択肢である。</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -12432,7 +12432,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>RFI（Request For Information：情報提供依頼書）は，発注者がITソリューションの提供者（ベンダー）に対して，導入検討の初期段階で活用事例や技術情報などの提供を依頼する文書である。したがって正解はウとなる。</t>
+          <t>RFI（Request For Information：情報提供依頼書）は，発注者がITソリューションの提供者（ベンダー）に対して，導入検討の初期段階で活用事例や技術情報などの提供を依頼する文書である。したがって正解は「RFI」である。</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -12517,7 +12517,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>IPランドスケープとは，事業・経営情報に知的財産（知財）情報を組み込んで分析し，現状の俯瞰や将来展望などの分析結果を事業責任者・経営者と共有して，事業戦略・経営戦略の立案に反映させる手法である。したがって正解はイとなる。</t>
+          <t>IPランドスケープとは，事業・経営情報に知的財産（知財）情報を組み込んで分析し，現状の俯瞰や将来展望などの分析結果を事業責任者・経営者と共有して，事業戦略・経営戦略の立案に反映させる手法である。したがって正解は「IPランドスケープ」である。</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
@@ -12602,7 +12602,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>カンパニー制組織は，一つの企業内に事業領域ごとに独立した「カンパニー」を設置し，各カンパニーに大幅な権限を委譲することで意思決定の迅速化と独立採算制を推進する組織形態である。したがって正解はアとなる。</t>
+          <t>カンパニー制組織は，一つの企業内に事業領域ごとに独立した「カンパニー」を設置し，各カンパニーに大幅な権限を委譲することで意思決定の迅速化と独立採算制を推進する組織形態である。したがって正解は「カンパニー制組織」である。</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -12690,7 +12690,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>不正アクセス禁止法では，他人の識別符号（ID・パスワード）を正当な理由なく本人に無断で第三者に提供する行為（識別符号提供罪，a），及び他人のID・パスワードを本人に無断で使用してサーバに不正にアクセスする行為（不正アクセス行為，c）が規制されている。一方，bのマルウェア作成行為は不正アクセス禁止法ではなく，不正指令電磁的記録に関する罪（刑法のウイルス作成罪）などで規制される行為であり，不正アクセス禁止法の直接の規制対象ではない。したがって，規制対象はaとcであり，正解はイとなる。</t>
+          <t>不正アクセス禁止法では，他人の識別符号（ID・パスワード）を正当な理由なく本人に無断で第三者に提供する行為（識別符号提供罪，a），及び他人のID・パスワードを本人に無断で使用してサーバに不正にアクセスする行為（不正アクセス行為，c）が規制されている。一方，bのマルウェア作成行為は不正アクセス禁止法ではなく，不正指令電磁的記録に関する罪（刑法のウイルス作成罪）などで規制される行為であり，不正アクセス禁止法の直接の規制対象ではない。したがって，規制対象はaとcであり，「a, c」を挙げている選択肢が正解となる。</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -12775,7 +12775,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>プロセスマイニングとは，業務システムの操作ログ（イベントログ）などの実績データを収集・分析し，実際に行われている業務プロセスを可視化・モニタリングすることで課題を特定し，改善につなげる手法・ツールである。したがって正解はアとなる。</t>
+          <t>プロセスマイニングとは，業務システムの操作ログ（イベントログ）などの実績データを収集・分析し，実際に行われている業務プロセスを可視化・モニタリングすることで課題を特定し，改善につなげる手法・ツールである。したがって正解は，業務の操作ログなどを収集し，業務プロセスの可視化・分析・モニタリングによって課題を特定して改善を図ると説明している選択肢である。</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -12860,7 +12860,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>アクセシビリティとは，高齢者や障害者を含む様々な能力・特性をもつ幅広い利用者が，等しく製品やサービスを利用できるように配慮された設計・状態を指す概念である。したがって正解はアとなる。</t>
+          <t>アクセシビリティとは，高齢者や障害者を含む様々な能力・特性をもつ幅広い利用者が，等しく製品やサービスを利用できるように配慮された設計・状態を指す概念である。したがって正解は，高齢者や障害者などを含め様々な能力や特性をもつ幅広い層の人が等しく利用できるように配慮した設計と説明している選択肢である。</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -12945,7 +12945,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>VR（Virtual Reality：仮想現実）は，ゴーグルなどの専用機器を用いて完全な仮想空間に没入する技術である。アはゴーグルを装着して仮想空間の映像に没入する防災訓練の事例であり，VRに該当する。イ・ウ・エは，いずれも現実の映像に仮想的な情報を重ね合わせるAR（拡張現実）の事例である。したがって正解はアとなる。</t>
+          <t>VR（Virtual Reality：仮想現実）は，ゴーグルなどの専用機器を用いて完全な仮想空間に没入する技術である。ゴーグルを装着して仮想空間の映像に没入する防災訓練の事例はVRに該当する。家具の試し置き，史跡の説明表示，図鑑の動画表示は，いずれも現実の映像に仮想的な情報を重ね合わせるAR（拡張現実）の事例である。したがって正解は，ゴーグルを装着して仮想空間の映像に没入する防災訓練の事例である。</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -13030,7 +13030,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>企画プロセスにおけるシステム化構想の立案段階では，どのような情報技術を活用できるかを把握するために，システム化する業務分野に関する情報技術動向をベンダー企業から収集することが重要である。したがって正解はイとなる。</t>
+          <t>企画プロセスにおけるシステム化構想の立案段階では，どのような情報技術を活用できるかを把握するために，システム化する業務分野に関する情報技術動向をベンダー企業から収集することが重要である。したがって正解は「システム化する業務の分野に関する情報技術動向」を挙げている選択肢である。</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -18507,7 +18507,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>PDCAモデルでは，P(Plan：計画)で目的や手順を定め，D(Do：実行)で手順に従って実施し，C(Check：評価)で第三者などによる客観的な評価を行い，A(Act：改善)で発見された問題点を是正する。作業(1)は目的・手順を定めるのでP，作業(3)は手順に従って監視を実行するのでD，作業(2)は第三者による評価なのでC，作業(4)は是正処置(監視方法の変更)なのでAに対応する。よってP=(1)，D=(3)，C=(2)，A=(4)となるウが正しい。</t>
+          <t>PDCAモデルでは，P(Plan：計画)で目的や手順を定め，D(Do：実行)で手順に従って実施し，C(Check：評価)で第三者などによる客観的な評価を行い，A(Act：改善)で発見された問題点を是正する。作業(1)は目的・手順を定めるのでP，作業(3)は手順に従って監視を実行するのでD，作業(2)は第三者による評価なのでC，作業(4)は是正処置(監視方法の変更)なのでAに対応する。よってP=(1)，D=(3)，C=(2)，A=(4)となる組合せ「(1)／(3)／(2)／(4)」が正しい。</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -26993,7 +26993,7 @@
       </c>
       <c r="M282" t="inlineStr">
         <is>
-          <t>正規化では，繰り返しや更新時異常を排除するため，項目間の関数従属性に着目して表を分割する。個数は「どの受注で何個注文したか」という受注に固有の値なので受注側の表に残す。一方，単価は商品番号によって一意に決まる（同一商品で単価が異なれば商品番号も別になる，という設問の前提）ため，商品番号・商品名とともに商品側の表にまとめるのが適切である。したがって，受注番号・発注者名・商品番号・個数を受注側，商品番号・商品名・単価を商品側に分けるエが正しい。</t>
+          <t>正規化では，繰り返しや更新時異常を排除するため，項目間の関数従属性に着目して表を分割する。個数は「どの受注で何個注文したか」という受注に固有の値なので受注側の表に残す。一方，単価は商品番号によって一意に決まる（同一商品で単価が異なれば商品番号も別になる，という設問の前提）ため，商品番号・商品名とともに商品側の表にまとめるのが適切である。したがって，受注番号・発注者名・商品番号・個数を受注側，商品番号・商品名・単価を商品側に分ける組合せが正しい。</t>
         </is>
       </c>
       <c r="N282" t="inlineStr">
@@ -33783,7 +33783,7 @@
       </c>
       <c r="M360" t="inlineStr">
         <is>
-          <t>会員番号は店舗ごとに付与されるため，会員番号だけでは一意に会員を特定できず，店舗コードと会員番号の組みで主キーとする必要がある。また，会員種別コードは会員ごとに異なる値を持つため（同じ会員でも登録店舗により会員種別が異なる例がある），会員表の非キー属性として残す必要がある。したがって，主キーを（会員番号，店舗コード），属性として会員名，会員種別コードをもつエが正しい。</t>
+          <t>会員番号は店舗ごとに付与されるため，会員番号だけでは一意に会員を特定できず，店舗コードと会員番号の組みで主キーとする必要がある。また，会員種別コードは会員ごとに異なる値を持つため（同じ会員でも登録店舗により会員種別が異なる例がある），会員表の非キー属性として残す必要がある。したがって，主キーを（会員番号，店舗コード），属性として会員名，会員種別コードをもつ選択肢が正しい。</t>
         </is>
       </c>
       <c r="N360" t="inlineStr">

</xml_diff>